<commit_message>
data viz structure done
</commit_message>
<xml_diff>
--- a/data/india_quick.xlsx
+++ b/data/india_quick.xlsx
@@ -8,17 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Self Development\Data Visualization\India - Quick Commerce\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F86C9B7-43B9-46E3-B3C5-F65918D65AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E36829-24F2-4150-8660-0996FBE6B0FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -93,17 +102,17 @@
     <t>Swiggy - Quick Commerce Share of Total Revenue</t>
   </si>
   <si>
-    <t>Zomato - Total revenue</t>
-  </si>
-  <si>
-    <t>Swiggy - Total revenue</t>
+    <t>Quarter Label</t>
+  </si>
+  <si>
+    <t>Quarter Index</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,25 +133,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -175,19 +172,15 @@
       <right style="medium">
         <color rgb="FFCCCCCC"/>
       </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFBFBFBF"/>
-      </bottom>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -201,20 +194,11 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -504,383 +488,410 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="6" t="s">
         <v>23</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5">
-        <v>1539</v>
+      <c r="B2" s="3">
+        <v>0.83399999999999996</v>
       </c>
       <c r="C2" s="3">
-        <v>0.83399999999999996</v>
-      </c>
-      <c r="D2" s="3">
         <v>0</v>
       </c>
+      <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="F2" t="str">
+        <f>LEFT(A2,2)</f>
+        <v>Q4</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5">
-        <v>1810</v>
+      <c r="B3" s="3">
+        <v>0.81200000000000006</v>
       </c>
       <c r="C3" s="3">
-        <v>0.81200000000000006</v>
-      </c>
-      <c r="D3" s="3">
         <v>0</v>
       </c>
+      <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F18" si="0">LEFT(A3,2)</f>
+        <v>Q1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5">
-        <v>2107</v>
+      <c r="B4" s="3">
+        <v>0.75</v>
       </c>
       <c r="C4" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="D4" s="3">
         <v>6.7000000000000004E-2</v>
       </c>
+      <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" t="str">
+        <f t="shared" si="0"/>
+        <v>Q2</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5">
-        <v>2363</v>
+      <c r="B5" s="3">
+        <v>0.66200000000000003</v>
       </c>
       <c r="C5" s="3">
-        <v>0.66200000000000003</v>
-      </c>
-      <c r="D5" s="3">
         <v>0.127</v>
       </c>
+      <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="F5" t="str">
+        <f t="shared" si="0"/>
+        <v>Q3</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="6">
-        <v>2413</v>
+      <c r="B6" s="3">
+        <v>0.63400000000000001</v>
       </c>
       <c r="C6" s="3">
-        <v>0.63400000000000001</v>
-      </c>
-      <c r="D6" s="3">
         <v>0.15</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" t="str">
+        <f t="shared" si="0"/>
+        <v>Q4</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="6">
-        <v>2786</v>
+      <c r="B7" s="3">
+        <v>0.625</v>
       </c>
       <c r="C7" s="3">
-        <v>0.625</v>
-      </c>
-      <c r="D7" s="3">
         <v>0.13800000000000001</v>
       </c>
-      <c r="E7" s="8">
-        <v>2694</v>
-      </c>
-      <c r="F7" s="4">
+      <c r="D7" s="4">
         <v>0.54</v>
       </c>
-      <c r="G7" s="4">
+      <c r="E7" s="4">
         <v>7.9000000000000001E-2</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="0"/>
+        <v>Q1</v>
+      </c>
+      <c r="G7">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6">
-        <v>3240</v>
+      <c r="B8" s="3">
+        <v>0.59799999999999998</v>
       </c>
       <c r="C8" s="3">
-        <v>0.59799999999999998</v>
-      </c>
-      <c r="D8" s="3">
         <v>0.156</v>
       </c>
-      <c r="E8" s="8">
-        <v>3061</v>
-      </c>
-      <c r="F8" s="4">
+      <c r="D8" s="4">
         <v>0.501</v>
       </c>
-      <c r="G8" s="4">
+      <c r="E8" s="4">
         <v>7.8E-2</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>Q2</v>
+      </c>
+      <c r="G8">
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="6">
-        <v>3646</v>
+      <c r="B9" s="3">
+        <v>0.56599999999999995</v>
       </c>
       <c r="C9" s="3">
-        <v>0.56599999999999995</v>
-      </c>
-      <c r="D9" s="3">
         <v>0.17699999999999999</v>
       </c>
-      <c r="E9" s="8">
-        <v>3298</v>
-      </c>
-      <c r="F9" s="4">
+      <c r="D9" s="4">
         <v>0.46500000000000002</v>
       </c>
-      <c r="G9" s="4">
+      <c r="E9" s="4">
         <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>Q3</v>
+      </c>
+      <c r="G9">
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="6">
-        <v>3873</v>
+      <c r="B10" s="3">
+        <v>0.52900000000000003</v>
       </c>
       <c r="C10" s="3">
-        <v>0.52900000000000003</v>
-      </c>
-      <c r="D10" s="3">
         <v>0.19900000000000001</v>
       </c>
-      <c r="E10" s="8">
-        <v>3268</v>
-      </c>
-      <c r="F10" s="4">
+      <c r="D10" s="4">
         <v>0.47699999999999998</v>
       </c>
-      <c r="G10" s="4">
+      <c r="E10" s="4">
         <v>0.105</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>Q4</v>
+      </c>
+      <c r="G10">
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="6">
-        <v>4520</v>
+      <c r="B11" s="3">
+        <v>0.499</v>
       </c>
       <c r="C11" s="3">
-        <v>0.499</v>
-      </c>
-      <c r="D11" s="3">
         <v>0.20799999999999999</v>
       </c>
-      <c r="E11" s="8">
-        <v>3477</v>
-      </c>
-      <c r="F11" s="4">
+      <c r="D11" s="4">
         <v>0.498</v>
       </c>
-      <c r="G11" s="4">
+      <c r="E11" s="4">
         <v>0.11600000000000001</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>Q1</v>
+      </c>
+      <c r="G11">
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="6">
-        <v>5127</v>
+      <c r="B12" s="3">
+        <v>0.45600000000000002</v>
       </c>
       <c r="C12" s="3">
-        <v>0.45600000000000002</v>
-      </c>
-      <c r="D12" s="3">
         <v>0.22500000000000001</v>
       </c>
-      <c r="E12" s="9">
-        <v>3873</v>
-      </c>
-      <c r="F12" s="4">
+      <c r="D12" s="4">
         <v>0.46700000000000003</v>
       </c>
-      <c r="G12" s="4">
+      <c r="E12" s="4">
         <v>0.13200000000000001</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="0"/>
+        <v>Q2</v>
+      </c>
+      <c r="G12">
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="6">
-        <v>5746</v>
+      <c r="B13" s="3">
+        <v>0.42</v>
       </c>
       <c r="C13" s="3">
-        <v>0.42</v>
-      </c>
-      <c r="D13" s="3">
         <v>0.24299999999999999</v>
       </c>
-      <c r="E13" s="9">
-        <v>4264</v>
-      </c>
-      <c r="F13" s="4">
+      <c r="D13" s="4">
         <v>0.436</v>
       </c>
-      <c r="G13" s="4">
+      <c r="E13" s="4">
         <v>0.14099999999999999</v>
+      </c>
+      <c r="F13" t="str">
+        <f t="shared" si="0"/>
+        <v>Q3</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="6">
-        <v>6188</v>
+      <c r="B14" s="3">
+        <v>0.38900000000000001</v>
       </c>
       <c r="C14" s="3">
-        <v>0.38900000000000001</v>
-      </c>
-      <c r="D14" s="3">
         <v>0.27600000000000002</v>
       </c>
-      <c r="E14" s="9">
-        <v>4718</v>
-      </c>
-      <c r="F14" s="4">
+      <c r="D14" s="4">
         <v>0.39600000000000002</v>
       </c>
-      <c r="G14" s="4">
+      <c r="E14" s="4">
         <v>0.155</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="0"/>
+        <v>Q4</v>
+      </c>
+      <c r="G14">
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="6">
-        <v>7563</v>
+      <c r="B15" s="3">
+        <v>0.35099999999999998</v>
       </c>
       <c r="C15" s="3">
-        <v>0.35099999999999998</v>
-      </c>
-      <c r="D15" s="3">
         <v>0.317</v>
       </c>
-      <c r="E15" s="9">
-        <v>5308</v>
-      </c>
-      <c r="F15" s="4">
+      <c r="D15" s="4">
         <v>0.39200000000000002</v>
       </c>
-      <c r="G15" s="4">
+      <c r="E15" s="4">
         <v>0.16200000000000001</v>
+      </c>
+      <c r="F15" t="str">
+        <f t="shared" si="0"/>
+        <v>Q1</v>
+      </c>
+      <c r="G15">
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="6">
-        <v>13968</v>
+      <c r="B16" s="3">
+        <v>0.20499999999999999</v>
       </c>
       <c r="C16" s="3">
-        <v>0.20499999999999999</v>
-      </c>
-      <c r="D16" s="3">
         <v>0.70799999999999996</v>
       </c>
-      <c r="E16" s="9">
-        <v>5911</v>
-      </c>
-      <c r="F16" s="4">
+      <c r="D16" s="4">
         <v>0.373</v>
       </c>
-      <c r="G16" s="4">
+      <c r="E16" s="4">
         <v>0.17599999999999999</v>
+      </c>
+      <c r="F16" t="str">
+        <f t="shared" si="0"/>
+        <v>Q2</v>
+      </c>
+      <c r="G16">
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="6">
-        <v>16692</v>
+      <c r="B17" s="3">
+        <v>0.183</v>
       </c>
       <c r="C17" s="3">
-        <v>0.183</v>
-      </c>
-      <c r="D17" s="3">
         <v>0.73399999999999999</v>
       </c>
-      <c r="E17" s="9">
-        <v>6431</v>
-      </c>
-      <c r="F17" s="4">
+      <c r="D17" s="4">
         <v>0.35399999999999998</v>
       </c>
-      <c r="G17" s="4">
+      <c r="E17" s="4">
         <v>0.16400000000000001</v>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" si="0"/>
+        <v>Q3</v>
+      </c>
+      <c r="G17">
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="6">
-        <v>17680</v>
+      <c r="B18" s="3">
+        <v>0.17699999999999999</v>
       </c>
       <c r="C18" s="3">
-        <v>0.17699999999999999</v>
-      </c>
-      <c r="D18" s="3">
         <v>0.748</v>
       </c>
-      <c r="E18" s="9">
-        <v>6665</v>
-      </c>
-      <c r="F18" s="4">
+      <c r="D18" s="4">
         <v>0.34599999999999997</v>
       </c>
-      <c r="G18" s="4">
+      <c r="E18" s="4">
         <v>0.16400000000000001</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="0"/>
+        <v>Q4</v>
+      </c>
+      <c r="G18">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
main data story axes complete
</commit_message>
<xml_diff>
--- a/data/india_quick.xlsx
+++ b/data/india_quick.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Self Development\Data Visualization\India - Quick Commerce\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E36829-24F2-4150-8660-0996FBE6B0FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3362D14D-CE21-40AA-A70C-D00AEF27CEC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
   <si>
     <t>Quarter</t>
   </si>
@@ -106,6 +106,18 @@
   </si>
   <si>
     <t>Quarter Index</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3</t>
   </si>
 </sst>
 </file>
@@ -180,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -195,9 +207,6 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -502,7 +511,7 @@
       <c r="F1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
     </row>
@@ -518,9 +527,8 @@
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" t="str">
-        <f>LEFT(A2,2)</f>
-        <v>Q4</v>
+      <c r="F2" t="s">
+        <v>24</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -538,9 +546,8 @@
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" t="str">
-        <f t="shared" ref="F3:F18" si="0">LEFT(A3,2)</f>
-        <v>Q1</v>
+      <c r="F3" t="s">
+        <v>25</v>
       </c>
       <c r="G3">
         <v>2</v>
@@ -558,9 +565,8 @@
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" t="str">
-        <f t="shared" si="0"/>
-        <v>Q2</v>
+      <c r="F4" t="s">
+        <v>26</v>
       </c>
       <c r="G4">
         <v>3</v>
@@ -578,9 +584,8 @@
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" t="str">
-        <f t="shared" si="0"/>
-        <v>Q3</v>
+      <c r="F5" t="s">
+        <v>27</v>
       </c>
       <c r="G5">
         <v>4</v>
@@ -598,9 +603,8 @@
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" t="str">
-        <f t="shared" si="0"/>
-        <v>Q4</v>
+      <c r="F6" t="s">
+        <v>24</v>
       </c>
       <c r="G6">
         <v>5</v>
@@ -622,9 +626,8 @@
       <c r="E7" s="4">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="F7" t="str">
-        <f t="shared" si="0"/>
-        <v>Q1</v>
+      <c r="F7" t="s">
+        <v>25</v>
       </c>
       <c r="G7">
         <v>6</v>
@@ -646,9 +649,8 @@
       <c r="E8" s="4">
         <v>7.8E-2</v>
       </c>
-      <c r="F8" t="str">
-        <f t="shared" si="0"/>
-        <v>Q2</v>
+      <c r="F8" t="s">
+        <v>26</v>
       </c>
       <c r="G8">
         <v>7</v>
@@ -670,9 +672,8 @@
       <c r="E9" s="4">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="F9" t="str">
-        <f t="shared" si="0"/>
-        <v>Q3</v>
+      <c r="F9" t="s">
+        <v>27</v>
       </c>
       <c r="G9">
         <v>8</v>
@@ -694,9 +695,8 @@
       <c r="E10" s="4">
         <v>0.105</v>
       </c>
-      <c r="F10" t="str">
-        <f t="shared" si="0"/>
-        <v>Q4</v>
+      <c r="F10" t="s">
+        <v>24</v>
       </c>
       <c r="G10">
         <v>9</v>
@@ -718,9 +718,8 @@
       <c r="E11" s="4">
         <v>0.11600000000000001</v>
       </c>
-      <c r="F11" t="str">
-        <f t="shared" si="0"/>
-        <v>Q1</v>
+      <c r="F11" t="s">
+        <v>25</v>
       </c>
       <c r="G11">
         <v>10</v>
@@ -742,9 +741,8 @@
       <c r="E12" s="4">
         <v>0.13200000000000001</v>
       </c>
-      <c r="F12" t="str">
-        <f t="shared" si="0"/>
-        <v>Q2</v>
+      <c r="F12" t="s">
+        <v>26</v>
       </c>
       <c r="G12">
         <v>11</v>
@@ -766,9 +764,8 @@
       <c r="E13" s="4">
         <v>0.14099999999999999</v>
       </c>
-      <c r="F13" t="str">
-        <f t="shared" si="0"/>
-        <v>Q3</v>
+      <c r="F13" t="s">
+        <v>27</v>
       </c>
       <c r="G13">
         <v>12</v>
@@ -790,9 +787,8 @@
       <c r="E14" s="4">
         <v>0.155</v>
       </c>
-      <c r="F14" t="str">
-        <f t="shared" si="0"/>
-        <v>Q4</v>
+      <c r="F14" t="s">
+        <v>24</v>
       </c>
       <c r="G14">
         <v>13</v>
@@ -814,9 +810,8 @@
       <c r="E15" s="4">
         <v>0.16200000000000001</v>
       </c>
-      <c r="F15" t="str">
-        <f t="shared" si="0"/>
-        <v>Q1</v>
+      <c r="F15" t="s">
+        <v>25</v>
       </c>
       <c r="G15">
         <v>14</v>
@@ -838,9 +833,8 @@
       <c r="E16" s="4">
         <v>0.17599999999999999</v>
       </c>
-      <c r="F16" t="str">
-        <f t="shared" si="0"/>
-        <v>Q2</v>
+      <c r="F16" t="s">
+        <v>26</v>
       </c>
       <c r="G16">
         <v>15</v>
@@ -862,9 +856,8 @@
       <c r="E17" s="4">
         <v>0.16400000000000001</v>
       </c>
-      <c r="F17" t="str">
-        <f t="shared" si="0"/>
-        <v>Q3</v>
+      <c r="F17" t="s">
+        <v>27</v>
       </c>
       <c r="G17">
         <v>16</v>
@@ -886,9 +879,8 @@
       <c r="E18" s="4">
         <v>0.16400000000000001</v>
       </c>
-      <c r="F18" t="str">
-        <f t="shared" si="0"/>
-        <v>Q4</v>
+      <c r="F18" t="s">
+        <v>24</v>
       </c>
       <c r="G18">
         <v>17</v>

</xml_diff>